<commit_message>
feat: expand curated innovation sources
</commit_message>
<xml_diff>
--- a/assets/innovation_news_ledger_template.xlsx
+++ b/assets/innovation_news_ledger_template.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R53aa1daf7c3d473c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="News Ledger" sheetId="2" r:id="Rc0f2b15893a94134"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source Registry" sheetId="3" r:id="R90b05928a184431b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Run Log" sheetId="4" r:id="R184c93856e664292"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R5dc8205e40c84459"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="News Ledger" sheetId="2" r:id="Rce9d125c23e14b82"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source Registry" sheetId="3" r:id="Rf82033ba313947a1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Run Log" sheetId="4" r:id="R61afd6ec1f16426f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -21,7 +21,7 @@
     <x:numFmt numFmtId="201" formatCode="0"/>
     <x:numFmt numFmtId="202" formatCode="yyyy-mm-dd hh:mm"/>
   </x:numFmts>
-  <x:fonts count="10">
+  <x:fonts count="12">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -76,8 +76,19 @@
       <x:color rgb="FFFFFFFF"/>
       <x:name val="DejaVu Sans"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:sz val="11"/>
+      <x:color rgb="FF1D2A35"/>
+      <x:name val="Carlito"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="8">
+  <x:fills count="14">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -114,8 +125,38 @@
         <x:fgColor rgb="FFF7ECD4"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF0F766E"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF0F766E"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF0F766E"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
-  <x:borders count="10">
+  <x:borders count="11">
     <x:border/>
     <x:border>
       <x:left style="thin">
@@ -198,11 +239,25 @@
         <x:color rgb="FF0B1F33"/>
       </x:bottom>
     </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFB8D6D0"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="FFB8D6D0"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFB8D6D0"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFB8D6D0"/>
+      </x:bottom>
+    </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="67">
+  <x:cellXfs count="98">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -359,6 +414,99 @@
     </x:xf>
     <x:xf numFmtId="200" fontId="4" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="8" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="8" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="9" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="9" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="9" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="9" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="9" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="9" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="10" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="11" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="11" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="11" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="11" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="11" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="11" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="12" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="13" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="13" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="13" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="13" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -398,9 +546,9 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="SourceRegistryTable" displayName="SourceRegistryTable" ref="A3:K37" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A3:K37"/>
-  <x:tableColumns count="11">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="SourceRegistryTable" displayName="SourceRegistryTable" ref="A3:N37" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A3:N37"/>
+  <x:tableColumns count="14">
     <x:tableColumn id="1" name="Active"/>
     <x:tableColumn id="2" name="Region"/>
     <x:tableColumn id="3" name="Country / Area"/>
@@ -412,6 +560,9 @@
     <x:tableColumn id="9" name="Priority"/>
     <x:tableColumn id="10" name="Native Feed"/>
     <x:tableColumn id="11" name="Notes"/>
+    <x:tableColumn id="12" name="Coverage Tier"/>
+    <x:tableColumn id="13" name="Cadence"/>
+    <x:tableColumn id="14" name="Topic Tags"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium4" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -768,7 +919,7 @@
         <x:v>Active sources</x:v>
       </x:c>
       <x:c r="B8" s="37" t="n">
-        <x:f>COUNTIF('Source Registry'!$A$4:$A$103,"Yes")</x:f>
+        <x:f>COUNTIF('Source Registry'!$A$4:$A$10003,"Yes")</x:f>
         <x:v>34</x:v>
       </x:c>
       <x:c r="C8" s="46"/>
@@ -1087,7 +1238,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf1d306d22e8b4f9c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9d7fde5df99c4b99"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1107,6 +1258,9 @@
     <x:col min="9" max="9" width="10" hidden="0" customWidth="1"/>
     <x:col min="10" max="10" width="13" hidden="0" customWidth="1"/>
     <x:col min="11" max="11" width="56" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="14" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="12" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="34" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="34" customHeight="1">
@@ -1126,7 +1280,7 @@
     </x:row>
     <x:row r="2" ht="25" customHeight="1">
       <x:c r="A2" s="13" t="str">
-        <x:v>Allowlist: government, official companies, major media, policy institutes, and leading journals</x:v>
+        <x:v>Allowlist: official/public sources and established media; S/A daily, B weekly; strict relevance on broad sources</x:v>
       </x:c>
       <x:c r="B2" s="14"/>
       <x:c r="C2" s="14"/>
@@ -1173,6 +1327,15 @@
       <x:c r="K3" s="59" t="str">
         <x:v>Notes</x:v>
       </x:c>
+      <x:c r="L3" s="93" t="str">
+        <x:v>Coverage Tier</x:v>
+      </x:c>
+      <x:c r="M3" s="93" t="str">
+        <x:v>Cadence</x:v>
+      </x:c>
+      <x:c r="N3" s="93" t="str">
+        <x:v>Topic Tags</x:v>
+      </x:c>
     </x:row>
     <x:row r="4" ht="42" customHeight="1">
       <x:c r="A4" s="60" t="str">
@@ -1208,6 +1371,13 @@
       <x:c r="K4" s="60" t="str">
         <x:v>Established global business and policy news.</x:v>
       </x:c>
+      <x:c r="L4" s="94" t="str">
+        <x:v>S</x:v>
+      </x:c>
+      <x:c r="M4" s="94" t="str">
+        <x:v>Daily</x:v>
+      </x:c>
+      <x:c r="N4" s="95" t="str"/>
     </x:row>
     <x:row r="5" ht="42" customHeight="1">
       <x:c r="A5" s="64" t="str">
@@ -1243,6 +1413,13 @@
       <x:c r="K5" s="64" t="str">
         <x:v>Broad science coverage; topic filter is applied.</x:v>
       </x:c>
+      <x:c r="L5" s="96" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="M5" s="96" t="str">
+        <x:v>Daily</x:v>
+      </x:c>
+      <x:c r="N5" s="97" t="str"/>
     </x:row>
     <x:row r="6" ht="42" customHeight="1">
       <x:c r="A6" s="64" t="str">
@@ -1278,6 +1455,13 @@
       <x:c r="K6" s="64" t="str">
         <x:v>Major media; strict topic filter is applied.</x:v>
       </x:c>
+      <x:c r="L6" s="96" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="M6" s="96" t="str">
+        <x:v>Weekly</x:v>
+      </x:c>
+      <x:c r="N6" s="97" t="str"/>
     </x:row>
     <x:row r="7" ht="42" customHeight="1">
       <x:c r="A7" s="64" t="str">
@@ -1313,6 +1497,13 @@
       <x:c r="K7" s="64" t="str">
         <x:v>Established specialist publication.</x:v>
       </x:c>
+      <x:c r="L7" s="96" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="M7" s="96" t="str">
+        <x:v>Daily</x:v>
+      </x:c>
+      <x:c r="N7" s="97" t="str"/>
     </x:row>
     <x:row r="8" ht="42" customHeight="1">
       <x:c r="A8" s="64" t="str">
@@ -1348,6 +1539,13 @@
       <x:c r="K8" s="64" t="str">
         <x:v>IEEE editorial publication.</x:v>
       </x:c>
+      <x:c r="L8" s="96" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="M8" s="96" t="str">
+        <x:v>Daily</x:v>
+      </x:c>
+      <x:c r="N8" s="97" t="str"/>
     </x:row>
     <x:row r="9" ht="42" customHeight="1">
       <x:c r="A9" s="64" t="str">
@@ -1383,6 +1581,13 @@
       <x:c r="K9" s="64" t="str">
         <x:v>Leading scientific publication; innovation-topic filter is applied.</x:v>
       </x:c>
+      <x:c r="L9" s="96" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="M9" s="96" t="str">
+        <x:v>Daily</x:v>
+      </x:c>
+      <x:c r="N9" s="97" t="str"/>
     </x:row>
     <x:row r="10" ht="42" customHeight="1">
       <x:c r="A10" s="64" t="str">
@@ -1418,6 +1623,13 @@
       <x:c r="K10" s="64" t="str">
         <x:v>Leading scientific publication; the publisher may rate-limit automated access.</x:v>
       </x:c>
+      <x:c r="L10" s="96" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="M10" s="96" t="str">
+        <x:v>Daily</x:v>
+      </x:c>
+      <x:c r="N10" s="97" t="str"/>
     </x:row>
     <x:row r="11" ht="42" customHeight="1">
       <x:c r="A11" s="64" t="str">
@@ -1453,6 +1665,13 @@
       <x:c r="K11" s="64" t="str">
         <x:v>Major Asia-focused media.</x:v>
       </x:c>
+      <x:c r="L11" s="96" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="M11" s="96" t="str">
+        <x:v>Daily</x:v>
+      </x:c>
+      <x:c r="N11" s="97" t="str"/>
     </x:row>
     <x:row r="12" ht="42" customHeight="1">
       <x:c r="A12" s="64" t="str">
@@ -1488,6 +1707,13 @@
       <x:c r="K12" s="64" t="str">
         <x:v>Established regional media; topic filter is applied.</x:v>
       </x:c>
+      <x:c r="L12" s="96" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="M12" s="96" t="str">
+        <x:v>Weekly</x:v>
+      </x:c>
+      <x:c r="N12" s="97" t="str"/>
     </x:row>
     <x:row r="13" ht="42" customHeight="1">
       <x:c r="A13" s="64" t="str">
@@ -1523,6 +1749,13 @@
       <x:c r="K13" s="64" t="str">
         <x:v>Established UAE-based regional newspaper; official technology feed.</x:v>
       </x:c>
+      <x:c r="L13" s="96" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="M13" s="96" t="str">
+        <x:v>Daily</x:v>
+      </x:c>
+      <x:c r="N13" s="97" t="str"/>
     </x:row>
     <x:row r="14" ht="42" customHeight="1">
       <x:c r="A14" s="64" t="str">
@@ -1558,6 +1791,13 @@
       <x:c r="K14" s="64" t="str">
         <x:v>Technology-policy analysis from Brookings; official listing-page fallback.</x:v>
       </x:c>
+      <x:c r="L14" s="96" t="str">
+        <x:v>S</x:v>
+      </x:c>
+      <x:c r="M14" s="96" t="str">
+        <x:v>Daily</x:v>
+      </x:c>
+      <x:c r="N14" s="97" t="str"/>
     </x:row>
     <x:row r="15" ht="42" customHeight="1">
       <x:c r="A15" s="64" t="str">
@@ -1593,6 +1833,13 @@
       <x:c r="K15" s="64" t="str">
         <x:v>Broad analysis feed; innovation-topic filter is applied.</x:v>
       </x:c>
+      <x:c r="L15" s="96" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="M15" s="96" t="str">
+        <x:v>Daily</x:v>
+      </x:c>
+      <x:c r="N15" s="97" t="str"/>
     </x:row>
     <x:row r="16" ht="42" customHeight="1">
       <x:c r="A16" s="64" t="str">
@@ -1628,6 +1875,13 @@
       <x:c r="K16" s="64" t="str">
         <x:v>University-based emerging-technology policy center.</x:v>
       </x:c>
+      <x:c r="L16" s="96" t="str">
+        <x:v>S</x:v>
+      </x:c>
+      <x:c r="M16" s="96" t="str">
+        <x:v>Daily</x:v>
+      </x:c>
+      <x:c r="N16" s="97" t="str"/>
     </x:row>
     <x:row r="17" ht="42" customHeight="1">
       <x:c r="A17" s="64" t="str">
@@ -1663,6 +1917,13 @@
       <x:c r="K17" s="64" t="str">
         <x:v>European economic-policy institute.</x:v>
       </x:c>
+      <x:c r="L17" s="96" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="M17" s="96" t="str">
+        <x:v>Daily</x:v>
+      </x:c>
+      <x:c r="N17" s="97" t="str"/>
     </x:row>
     <x:row r="18" ht="42" customHeight="1">
       <x:c r="A18" s="64" t="str">
@@ -1698,6 +1959,13 @@
       <x:c r="K18" s="64" t="str">
         <x:v>China-focused policy institute.</x:v>
       </x:c>
+      <x:c r="L18" s="96" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="M18" s="96" t="str">
+        <x:v>Daily</x:v>
+      </x:c>
+      <x:c r="N18" s="97" t="str"/>
     </x:row>
     <x:row r="19" ht="42" customHeight="1">
       <x:c r="A19" s="64" t="str">
@@ -1733,6 +2001,13 @@
       <x:c r="K19" s="64" t="str">
         <x:v>Official U.S. government source.</x:v>
       </x:c>
+      <x:c r="L19" s="96" t="str">
+        <x:v>S</x:v>
+      </x:c>
+      <x:c r="M19" s="96" t="str">
+        <x:v>Daily</x:v>
+      </x:c>
+      <x:c r="N19" s="97" t="str"/>
     </x:row>
     <x:row r="20" ht="42" customHeight="1">
       <x:c r="A20" s="64" t="str">
@@ -1768,6 +2043,13 @@
       <x:c r="K20" s="64" t="str">
         <x:v>Official U.S. government source.</x:v>
       </x:c>
+      <x:c r="L20" s="96" t="str">
+        <x:v>S</x:v>
+      </x:c>
+      <x:c r="M20" s="96" t="str">
+        <x:v>Daily</x:v>
+      </x:c>
+      <x:c r="N20" s="97" t="str"/>
     </x:row>
     <x:row r="21" ht="42" customHeight="1">
       <x:c r="A21" s="64" t="str">
@@ -1803,6 +2085,15 @@
       <x:c r="K21" s="64" t="str">
         <x:v>Official U.S. biomedical-research source.</x:v>
       </x:c>
+      <x:c r="L21" s="96" t="str">
+        <x:v>S</x:v>
+      </x:c>
+      <x:c r="M21" s="96" t="str">
+        <x:v>Daily</x:v>
+      </x:c>
+      <x:c r="N21" s="97" t="str">
+        <x:v>Biotechnology | Healthcare</x:v>
+      </x:c>
     </x:row>
     <x:row r="22" ht="42" customHeight="1">
       <x:c r="A22" s="64" t="str">
@@ -1838,6 +2129,15 @@
       <x:c r="K22" s="64" t="str">
         <x:v>Official U.S. government source; includes fusion and quantum policy.</x:v>
       </x:c>
+      <x:c r="L22" s="96" t="str">
+        <x:v>S</x:v>
+      </x:c>
+      <x:c r="M22" s="96" t="str">
+        <x:v>Daily</x:v>
+      </x:c>
+      <x:c r="N22" s="97" t="str">
+        <x:v>Quantum</x:v>
+      </x:c>
     </x:row>
     <x:row r="23" ht="42" customHeight="1">
       <x:c r="A23" s="64" t="str">
@@ -1873,6 +2173,13 @@
       <x:c r="K23" s="64" t="str">
         <x:v>Official European Commission press releases.</x:v>
       </x:c>
+      <x:c r="L23" s="96" t="str">
+        <x:v>S</x:v>
+      </x:c>
+      <x:c r="M23" s="96" t="str">
+        <x:v>Daily</x:v>
+      </x:c>
+      <x:c r="N23" s="97" t="str"/>
     </x:row>
     <x:row r="24" ht="42" customHeight="1">
       <x:c r="A24" s="64" t="str">
@@ -1908,6 +2215,13 @@
       <x:c r="K24" s="64" t="str">
         <x:v>Official UK government Atom feed.</x:v>
       </x:c>
+      <x:c r="L24" s="96" t="str">
+        <x:v>S</x:v>
+      </x:c>
+      <x:c r="M24" s="96" t="str">
+        <x:v>Daily</x:v>
+      </x:c>
+      <x:c r="N24" s="97" t="str"/>
     </x:row>
     <x:row r="25" ht="42" customHeight="1">
       <x:c r="A25" s="64" t="str">
@@ -1943,6 +2257,13 @@
       <x:c r="K25" s="64" t="str">
         <x:v>Official Japanese government English-language feed.</x:v>
       </x:c>
+      <x:c r="L25" s="96" t="str">
+        <x:v>S</x:v>
+      </x:c>
+      <x:c r="M25" s="96" t="str">
+        <x:v>Daily</x:v>
+      </x:c>
+      <x:c r="N25" s="97" t="str"/>
     </x:row>
     <x:row r="26" ht="42" customHeight="1">
       <x:c r="A26" s="64" t="str">
@@ -1978,6 +2299,15 @@
       <x:c r="K26" s="64" t="str">
         <x:v>Official international public-health source.</x:v>
       </x:c>
+      <x:c r="L26" s="96" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="M26" s="96" t="str">
+        <x:v>Daily</x:v>
+      </x:c>
+      <x:c r="N26" s="97" t="str">
+        <x:v>Healthcare</x:v>
+      </x:c>
     </x:row>
     <x:row r="27" ht="42" customHeight="1">
       <x:c r="A27" s="64" t="str">
@@ -2013,6 +2343,13 @@
       <x:c r="K27" s="64" t="str">
         <x:v>Official international energy-policy source.</x:v>
       </x:c>
+      <x:c r="L27" s="96" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="M27" s="96" t="str">
+        <x:v>Daily</x:v>
+      </x:c>
+      <x:c r="N27" s="97" t="str"/>
     </x:row>
     <x:row r="28" ht="42" customHeight="1">
       <x:c r="A28" s="64" t="str">
@@ -2048,6 +2385,13 @@
       <x:c r="K28" s="64" t="str">
         <x:v>Official OECD source.</x:v>
       </x:c>
+      <x:c r="L28" s="96" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="M28" s="96" t="str">
+        <x:v>Daily</x:v>
+      </x:c>
+      <x:c r="N28" s="97" t="str"/>
     </x:row>
     <x:row r="29" ht="42" customHeight="1">
       <x:c r="A29" s="64" t="str">
@@ -2083,6 +2427,15 @@
       <x:c r="K29" s="64" t="str">
         <x:v>Official company newsroom.</x:v>
       </x:c>
+      <x:c r="L29" s="96" t="str">
+        <x:v>S</x:v>
+      </x:c>
+      <x:c r="M29" s="96" t="str">
+        <x:v>Daily</x:v>
+      </x:c>
+      <x:c r="N29" s="97" t="str">
+        <x:v>Artificial Intelligence</x:v>
+      </x:c>
     </x:row>
     <x:row r="30" ht="42" customHeight="1">
       <x:c r="A30" s="64" t="str">
@@ -2118,6 +2471,15 @@
       <x:c r="K30" s="64" t="str">
         <x:v>Official company publication.</x:v>
       </x:c>
+      <x:c r="L30" s="96" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="M30" s="96" t="str">
+        <x:v>Daily</x:v>
+      </x:c>
+      <x:c r="N30" s="97" t="str">
+        <x:v>Artificial Intelligence</x:v>
+      </x:c>
     </x:row>
     <x:row r="31" ht="42" customHeight="1">
       <x:c r="A31" s="64" t="str">
@@ -2153,6 +2515,15 @@
       <x:c r="K31" s="64" t="str">
         <x:v>Official company publication.</x:v>
       </x:c>
+      <x:c r="L31" s="96" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="M31" s="96" t="str">
+        <x:v>Daily</x:v>
+      </x:c>
+      <x:c r="N31" s="97" t="str">
+        <x:v>Artificial Intelligence | Semiconductors &amp; Telecom</x:v>
+      </x:c>
     </x:row>
     <x:row r="32" ht="42" customHeight="1">
       <x:c r="A32" s="64" t="str">
@@ -2188,6 +2559,15 @@
       <x:c r="K32" s="64" t="str">
         <x:v>Official company newsroom.</x:v>
       </x:c>
+      <x:c r="L32" s="96" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="M32" s="96" t="str">
+        <x:v>Daily</x:v>
+      </x:c>
+      <x:c r="N32" s="97" t="str">
+        <x:v>Semiconductors &amp; Telecom</x:v>
+      </x:c>
     </x:row>
     <x:row r="33" ht="42" customHeight="1">
       <x:c r="A33" s="64" t="str">
@@ -2223,6 +2603,15 @@
       <x:c r="K33" s="64" t="str">
         <x:v>Official corporate research publication.</x:v>
       </x:c>
+      <x:c r="L33" s="96" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="M33" s="96" t="str">
+        <x:v>Daily</x:v>
+      </x:c>
+      <x:c r="N33" s="97" t="str">
+        <x:v>Artificial Intelligence | Quantum</x:v>
+      </x:c>
     </x:row>
     <x:row r="34" ht="42" customHeight="1">
       <x:c r="A34" s="64" t="str">
@@ -2258,6 +2647,15 @@
       <x:c r="K34" s="64" t="str">
         <x:v>Official corporate research publication.</x:v>
       </x:c>
+      <x:c r="L34" s="96" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="M34" s="96" t="str">
+        <x:v>Daily</x:v>
+      </x:c>
+      <x:c r="N34" s="97" t="str">
+        <x:v>Artificial Intelligence | Quantum</x:v>
+      </x:c>
     </x:row>
     <x:row r="35" ht="42" customHeight="1">
       <x:c r="A35" s="64" t="str">
@@ -2293,6 +2691,15 @@
       <x:c r="K35" s="64" t="str">
         <x:v>Official company newsroom.</x:v>
       </x:c>
+      <x:c r="L35" s="96" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="M35" s="96" t="str">
+        <x:v>Daily</x:v>
+      </x:c>
+      <x:c r="N35" s="97" t="str">
+        <x:v>Artificial Intelligence | Semiconductors &amp; Telecom</x:v>
+      </x:c>
     </x:row>
     <x:row r="36" ht="42" customHeight="1">
       <x:c r="A36" s="64" t="str">
@@ -2328,6 +2735,15 @@
       <x:c r="K36" s="64" t="str">
         <x:v>Official international fusion project; official listing-page fallback.</x:v>
       </x:c>
+      <x:c r="L36" s="96" t="str">
+        <x:v>S</x:v>
+      </x:c>
+      <x:c r="M36" s="96" t="str">
+        <x:v>Daily</x:v>
+      </x:c>
+      <x:c r="N36" s="97" t="str">
+        <x:v>Fusion Energy</x:v>
+      </x:c>
     </x:row>
     <x:row r="37" ht="42" customHeight="1">
       <x:c r="A37" s="64" t="str">
@@ -2363,11 +2779,20 @@
       <x:c r="K37" s="64" t="str">
         <x:v>Established industry association; company claims are clearly labeled by source.</x:v>
       </x:c>
+      <x:c r="L37" s="96" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="M37" s="96" t="str">
+        <x:v>Weekly</x:v>
+      </x:c>
+      <x:c r="N37" s="97" t="str">
+        <x:v>Fusion Energy</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
-    <x:mergeCell ref="A1:K1"/>
-    <x:mergeCell ref="A2:K2"/>
+    <x:mergeCell ref="A1:N1"/>
+    <x:mergeCell ref="A2:N2"/>
   </x:mergeCells>
   <x:dataValidations count="1">
     <x:dataValidation type="list" sqref="A4:A37">
@@ -2376,7 +2801,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R14da59c788c1430f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8ea3cfa159444d8f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2462,7 +2887,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra3b574e118a544f5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfd098bede6154a30"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>